<commit_message>
Edits on pelagic species
</commit_message>
<xml_diff>
--- a/Data/Nutritional_database.xlsx
+++ b/Data/Nutritional_database.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/victorbrun/Documents/travail/These/Travaux/Food SFB/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAED566A-5C50-C84E-924F-DB54A0C1943C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31D232E1-65C4-6C4C-8F5E-BA2643607CC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1200" windowWidth="25600" windowHeight="15260" xr2:uid="{8C7B3EC4-DD38-D645-B1C5-87DFD8FAF630}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16640" xr2:uid="{8C7B3EC4-DD38-D645-B1C5-87DFD8FAF630}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$P$1</definedName>
@@ -29,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="361">
   <si>
     <t>Leaves_kamote</t>
   </si>
@@ -1109,6 +1108,9 @@
   </si>
   <si>
     <t>last three blood sausage</t>
+  </si>
+  <si>
+    <t>Soft bottom</t>
   </si>
 </sst>
 </file>
@@ -1639,9 +1641,6 @@
       <c r="B4" t="s">
         <v>277</v>
       </c>
-      <c r="C4" t="s">
-        <v>174</v>
-      </c>
       <c r="D4" t="s">
         <v>275</v>
       </c>
@@ -1686,9 +1685,6 @@
       <c r="B5" t="s">
         <v>280</v>
       </c>
-      <c r="C5" t="s">
-        <v>174</v>
-      </c>
       <c r="D5" t="s">
         <v>275</v>
       </c>
@@ -2781,7 +2777,7 @@
         <v>193</v>
       </c>
       <c r="C33" t="s">
-        <v>174</v>
+        <v>360</v>
       </c>
       <c r="D33" t="s">
         <v>275</v>
@@ -2941,6 +2937,9 @@
       <c r="B37" t="s">
         <v>167</v>
       </c>
+      <c r="C37" t="s">
+        <v>175</v>
+      </c>
       <c r="D37" t="s">
         <v>275</v>
       </c>
@@ -2973,6 +2972,9 @@
       <c r="B38" t="s">
         <v>337</v>
       </c>
+      <c r="C38" t="s">
+        <v>176</v>
+      </c>
       <c r="D38" t="s">
         <v>275</v>
       </c>
@@ -4178,7 +4180,7 @@
         <v>357</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>174</v>
+        <v>360</v>
       </c>
       <c r="D67" t="s">
         <v>275</v>
@@ -4295,7 +4297,7 @@
         <v>206</v>
       </c>
       <c r="C70" t="s">
-        <v>174</v>
+        <v>360</v>
       </c>
       <c r="D70" t="s">
         <v>275</v>
@@ -4696,7 +4698,7 @@
         <v>210</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>174</v>
+        <v>360</v>
       </c>
       <c r="D80" t="s">
         <v>275</v>
@@ -5026,6 +5028,9 @@
       <c r="B88" t="s">
         <v>296</v>
       </c>
+      <c r="C88" t="s">
+        <v>175</v>
+      </c>
       <c r="D88" t="s">
         <v>275</v>
       </c>
@@ -5571,6 +5576,9 @@
       <c r="B101" t="s">
         <v>199</v>
       </c>
+      <c r="C101" t="s">
+        <v>174</v>
+      </c>
       <c r="D101" t="s">
         <v>275</v>
       </c>
@@ -5966,6 +5974,9 @@
       </c>
       <c r="B111" t="s">
         <v>225</v>
+      </c>
+      <c r="C111" t="s">
+        <v>174</v>
       </c>
       <c r="D111" t="s">
         <v>275</v>
@@ -6570,6 +6581,9 @@
       <c r="B126" t="s">
         <v>236</v>
       </c>
+      <c r="C126" t="s">
+        <v>176</v>
+      </c>
       <c r="D126" t="s">
         <v>275</v>
       </c>
@@ -7496,7 +7510,7 @@
         <v>246</v>
       </c>
       <c r="C149" t="s">
-        <v>174</v>
+        <v>360</v>
       </c>
       <c r="D149" t="s">
         <v>275</v>
@@ -7665,6 +7679,9 @@
       <c r="B153" t="s">
         <v>248</v>
       </c>
+      <c r="C153" t="s">
+        <v>174</v>
+      </c>
       <c r="D153" t="s">
         <v>275</v>
       </c>
@@ -8124,6 +8141,9 @@
       </c>
       <c r="B164" t="s">
         <v>356</v>
+      </c>
+      <c r="C164" t="s">
+        <v>174</v>
       </c>
       <c r="D164" t="s">
         <v>275</v>
@@ -8750,13 +8770,4 @@
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7857BAE7-01AA-FA49-94C7-4551CCEF7345}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>